<commit_message>
Update 3-set match system
</commit_message>
<xml_diff>
--- a/backend/data/results.xlsx
+++ b/backend/data/results.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경기결과" sheetId="1" r:id="Rb21a66059e3e4772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경기결과" sheetId="1" r:id="R32d4db0f9f9148e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -28,7 +29,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -42,13 +43,70 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF3CD"/>
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F4F6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="18">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD2DC"/>
+      </x:bottom>
+    </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFCBD2DC"/>
@@ -105,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -124,19 +182,35 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -150,32 +224,107 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -185,13 +334,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsTable" displayName="ResultsTable" ref="A1:E21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MatchResults3SetsTable" displayName="MatchResults3SetsTable" ref="A1:I21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
     <x:tableColumn id="1" name="경기 날짜"/>
     <x:tableColumn id="2" name="팀A"/>
-    <x:tableColumn id="3" name="팀A 점수"/>
-    <x:tableColumn id="4" name="팀B 점수"/>
-    <x:tableColumn id="5" name="팀B"/>
+    <x:tableColumn id="3" name="1세트 팀A 득점"/>
+    <x:tableColumn id="4" name="1세트 팀B 득점"/>
+    <x:tableColumn id="5" name="2세트 팀A 득점"/>
+    <x:tableColumn id="6" name="2세트 팀B 득점"/>
+    <x:tableColumn id="7" name="3세트 팀A 득점"/>
+    <x:tableColumn id="8" name="3세트 팀B 득점"/>
+    <x:tableColumn id="9" name="팀B"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -392,294 +545,420 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="22" customHeight="1">
-      <x:c r="A1" s="20" t="str">
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="26" t="str">
         <x:v>경기 날짜</x:v>
       </x:c>
-      <x:c r="B1" s="21" t="str">
+      <x:c r="B1" s="27" t="str">
         <x:v>팀A</x:v>
       </x:c>
-      <x:c r="C1" s="21" t="str">
-        <x:v>팀A 점수</x:v>
-      </x:c>
-      <x:c r="D1" s="21" t="str">
-        <x:v>팀B 점수</x:v>
-      </x:c>
-      <x:c r="E1" s="22" t="str">
+      <x:c r="C1" s="27" t="str">
+        <x:v>1세트 팀A 득점</x:v>
+      </x:c>
+      <x:c r="D1" s="27" t="str">
+        <x:v>1세트 팀B 득점</x:v>
+      </x:c>
+      <x:c r="E1" s="27" t="str">
+        <x:v>2세트 팀A 득점</x:v>
+      </x:c>
+      <x:c r="F1" s="27" t="str">
+        <x:v>2세트 팀B 득점</x:v>
+      </x:c>
+      <x:c r="G1" s="27" t="str">
+        <x:v>3세트 팀A 득점</x:v>
+      </x:c>
+      <x:c r="H1" s="27" t="str">
+        <x:v>3세트 팀B 득점</x:v>
+      </x:c>
+      <x:c r="I1" s="28" t="str">
         <x:v>팀B</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="23" t="n">
+      <x:c r="K1" s="6" t="str">
+        <x:v>입력 규칙</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="29" t="n">
         <x:v>46270</x:v>
       </x:c>
-      <x:c r="B2" s="13" t="str">
+      <x:c r="B2" s="18" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C2" s="18"/>
-      <x:c r="D2" s="18"/>
-      <x:c r="E2" s="24" t="str">
+      <x:c r="C2" s="24"/>
+      <x:c r="D2" s="24"/>
+      <x:c r="E2" s="24"/>
+      <x:c r="F2" s="24"/>
+      <x:c r="G2" s="24"/>
+      <x:c r="H2" s="24"/>
+      <x:c r="I2" s="30" t="str">
         <x:v>이준석</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="23" t="n">
+      <x:c r="K2" s="50" t="str">
+        <x:v>• 승패와 관계없이 매 경기 3세트 진행
+• 3세트 모두 승점 계산 대상
+• 노란색 칸에 각 세트의 실제 득점 입력
+• 한 참가자당 정규리그 8경기 = 총 24세트</x:v>
+      </x:c>
+      <x:c r="L2" s="51"/>
+      <x:c r="M2" s="52"/>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="29" t="n">
         <x:v>46270</x:v>
       </x:c>
-      <x:c r="B3" s="13" t="str">
+      <x:c r="B3" s="18" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C3" s="18"/>
-      <x:c r="D3" s="18"/>
-      <x:c r="E3" s="24" t="str">
+      <x:c r="C3" s="24"/>
+      <x:c r="D3" s="24"/>
+      <x:c r="E3" s="24"/>
+      <x:c r="F3" s="24"/>
+      <x:c r="G3" s="24"/>
+      <x:c r="H3" s="24"/>
+      <x:c r="I3" s="30" t="str">
         <x:v>이상</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="22" customHeight="1">
-      <x:c r="A4" s="23" t="n">
+      <x:c r="K3" s="53"/>
+      <x:c r="L3" s="48"/>
+      <x:c r="M3" s="54"/>
+    </x:row>
+    <x:row r="4" ht="25" customHeight="1">
+      <x:c r="A4" s="29" t="n">
         <x:v>46271</x:v>
       </x:c>
-      <x:c r="B4" s="13" t="str">
+      <x:c r="B4" s="18" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C4" s="18"/>
-      <x:c r="D4" s="18"/>
-      <x:c r="E4" s="24" t="str">
+      <x:c r="C4" s="24"/>
+      <x:c r="D4" s="24"/>
+      <x:c r="E4" s="24"/>
+      <x:c r="F4" s="24"/>
+      <x:c r="G4" s="24"/>
+      <x:c r="H4" s="24"/>
+      <x:c r="I4" s="30" t="str">
         <x:v>문권기</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="22" customHeight="1">
-      <x:c r="A5" s="23" t="n">
+      <x:c r="K4" s="53"/>
+      <x:c r="L4" s="48"/>
+      <x:c r="M4" s="54"/>
+    </x:row>
+    <x:row r="5" ht="25" customHeight="1">
+      <x:c r="A5" s="29" t="n">
         <x:v>46271</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="str">
+      <x:c r="B5" s="18" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C5" s="18"/>
-      <x:c r="D5" s="18"/>
-      <x:c r="E5" s="24" t="str">
+      <x:c r="C5" s="24"/>
+      <x:c r="D5" s="24"/>
+      <x:c r="E5" s="24"/>
+      <x:c r="F5" s="24"/>
+      <x:c r="G5" s="24"/>
+      <x:c r="H5" s="24"/>
+      <x:c r="I5" s="30" t="str">
         <x:v>이준석</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="22" customHeight="1">
-      <x:c r="A6" s="23" t="n">
+      <x:c r="K5" s="53"/>
+      <x:c r="L5" s="48"/>
+      <x:c r="M5" s="54"/>
+    </x:row>
+    <x:row r="6" ht="25" customHeight="1">
+      <x:c r="A6" s="29" t="n">
         <x:v>46277</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="str">
+      <x:c r="B6" s="18" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C6" s="18"/>
-      <x:c r="D6" s="18"/>
-      <x:c r="E6" s="24" t="str">
+      <x:c r="C6" s="24"/>
+      <x:c r="D6" s="24"/>
+      <x:c r="E6" s="24"/>
+      <x:c r="F6" s="24"/>
+      <x:c r="G6" s="24"/>
+      <x:c r="H6" s="24"/>
+      <x:c r="I6" s="30" t="str">
         <x:v>이상</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="22" customHeight="1">
-      <x:c r="A7" s="23" t="n">
+      <x:c r="K6" s="55"/>
+      <x:c r="L6" s="56"/>
+      <x:c r="M6" s="57"/>
+    </x:row>
+    <x:row r="7" ht="25" customHeight="1">
+      <x:c r="A7" s="29" t="n">
         <x:v>46277</x:v>
       </x:c>
-      <x:c r="B7" s="13" t="str">
+      <x:c r="B7" s="18" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C7" s="18"/>
-      <x:c r="D7" s="18"/>
-      <x:c r="E7" s="24" t="str">
+      <x:c r="C7" s="24"/>
+      <x:c r="D7" s="24"/>
+      <x:c r="E7" s="24"/>
+      <x:c r="F7" s="24"/>
+      <x:c r="G7" s="24"/>
+      <x:c r="H7" s="24"/>
+      <x:c r="I7" s="30" t="str">
         <x:v>서종원</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="22" customHeight="1">
-      <x:c r="A8" s="23" t="n">
+    <x:row r="8" ht="25" customHeight="1">
+      <x:c r="A8" s="29" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="str">
+      <x:c r="B8" s="18" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C8" s="18"/>
-      <x:c r="D8" s="18"/>
-      <x:c r="E8" s="24" t="str">
+      <x:c r="C8" s="24"/>
+      <x:c r="D8" s="24"/>
+      <x:c r="E8" s="24"/>
+      <x:c r="F8" s="24"/>
+      <x:c r="G8" s="24"/>
+      <x:c r="H8" s="24"/>
+      <x:c r="I8" s="30" t="str">
         <x:v>문권기</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="22" customHeight="1">
-      <x:c r="A9" s="23" t="n">
+    <x:row r="9" ht="25" customHeight="1">
+      <x:c r="A9" s="29" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="B9" s="13" t="str">
+      <x:c r="B9" s="18" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C9" s="18"/>
-      <x:c r="D9" s="18"/>
-      <x:c r="E9" s="24" t="str">
+      <x:c r="C9" s="24"/>
+      <x:c r="D9" s="24"/>
+      <x:c r="E9" s="24"/>
+      <x:c r="F9" s="24"/>
+      <x:c r="G9" s="24"/>
+      <x:c r="H9" s="24"/>
+      <x:c r="I9" s="30" t="str">
         <x:v>이준석</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="22" customHeight="1">
-      <x:c r="A10" s="23" t="n">
+    <x:row r="10" ht="25" customHeight="1">
+      <x:c r="A10" s="29" t="n">
         <x:v>46284</x:v>
       </x:c>
-      <x:c r="B10" s="13" t="str">
+      <x:c r="B10" s="18" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C10" s="18"/>
-      <x:c r="D10" s="18"/>
-      <x:c r="E10" s="24" t="str">
+      <x:c r="C10" s="24"/>
+      <x:c r="D10" s="24"/>
+      <x:c r="E10" s="24"/>
+      <x:c r="F10" s="24"/>
+      <x:c r="G10" s="24"/>
+      <x:c r="H10" s="24"/>
+      <x:c r="I10" s="30" t="str">
         <x:v>이준석</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="23" t="n">
+    <x:row r="11" ht="25" customHeight="1">
+      <x:c r="A11" s="29" t="n">
         <x:v>46284</x:v>
       </x:c>
-      <x:c r="B11" s="13" t="str">
+      <x:c r="B11" s="18" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C11" s="18"/>
-      <x:c r="D11" s="18"/>
-      <x:c r="E11" s="24" t="str">
+      <x:c r="C11" s="24"/>
+      <x:c r="D11" s="24"/>
+      <x:c r="E11" s="24"/>
+      <x:c r="F11" s="24"/>
+      <x:c r="G11" s="24"/>
+      <x:c r="H11" s="24"/>
+      <x:c r="I11" s="30" t="str">
         <x:v>서종원</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="23" t="n">
+    <x:row r="12" ht="25" customHeight="1">
+      <x:c r="A12" s="29" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="B12" s="13" t="str">
+      <x:c r="B12" s="18" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C12" s="18"/>
-      <x:c r="D12" s="18"/>
-      <x:c r="E12" s="24" t="str">
+      <x:c r="C12" s="24"/>
+      <x:c r="D12" s="24"/>
+      <x:c r="E12" s="24"/>
+      <x:c r="F12" s="24"/>
+      <x:c r="G12" s="24"/>
+      <x:c r="H12" s="24"/>
+      <x:c r="I12" s="30" t="str">
         <x:v>서종원</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="23" t="n">
+    <x:row r="13" ht="25" customHeight="1">
+      <x:c r="A13" s="29" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="B13" s="13" t="str">
+      <x:c r="B13" s="18" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C13" s="18"/>
-      <x:c r="D13" s="18"/>
-      <x:c r="E13" s="24" t="str">
+      <x:c r="C13" s="24"/>
+      <x:c r="D13" s="24"/>
+      <x:c r="E13" s="24"/>
+      <x:c r="F13" s="24"/>
+      <x:c r="G13" s="24"/>
+      <x:c r="H13" s="24"/>
+      <x:c r="I13" s="30" t="str">
         <x:v>주은성</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="23" t="n">
+    <x:row r="14" ht="25" customHeight="1">
+      <x:c r="A14" s="29" t="n">
         <x:v>46291</x:v>
       </x:c>
-      <x:c r="B14" s="13" t="str">
+      <x:c r="B14" s="18" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C14" s="18"/>
-      <x:c r="D14" s="18"/>
-      <x:c r="E14" s="24" t="str">
+      <x:c r="C14" s="24"/>
+      <x:c r="D14" s="24"/>
+      <x:c r="E14" s="24"/>
+      <x:c r="F14" s="24"/>
+      <x:c r="G14" s="24"/>
+      <x:c r="H14" s="24"/>
+      <x:c r="I14" s="30" t="str">
         <x:v>서종원</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="23" t="n">
+    <x:row r="15" ht="25" customHeight="1">
+      <x:c r="A15" s="29" t="n">
         <x:v>46291</x:v>
       </x:c>
-      <x:c r="B15" s="13" t="str">
+      <x:c r="B15" s="18" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C15" s="18"/>
-      <x:c r="D15" s="18"/>
-      <x:c r="E15" s="24" t="str">
+      <x:c r="C15" s="24"/>
+      <x:c r="D15" s="24"/>
+      <x:c r="E15" s="24"/>
+      <x:c r="F15" s="24"/>
+      <x:c r="G15" s="24"/>
+      <x:c r="H15" s="24"/>
+      <x:c r="I15" s="30" t="str">
         <x:v>주은성</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="22" customHeight="1">
-      <x:c r="A16" s="23" t="n">
+    <x:row r="16" ht="25" customHeight="1">
+      <x:c r="A16" s="29" t="n">
         <x:v>46292</x:v>
       </x:c>
-      <x:c r="B16" s="13" t="str">
+      <x:c r="B16" s="18" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C16" s="18"/>
-      <x:c r="D16" s="18"/>
-      <x:c r="E16" s="24" t="str">
+      <x:c r="C16" s="24"/>
+      <x:c r="D16" s="24"/>
+      <x:c r="E16" s="24"/>
+      <x:c r="F16" s="24"/>
+      <x:c r="G16" s="24"/>
+      <x:c r="H16" s="24"/>
+      <x:c r="I16" s="30" t="str">
         <x:v>문권기</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="22" customHeight="1">
-      <x:c r="A17" s="23" t="n">
+    <x:row r="17" ht="25" customHeight="1">
+      <x:c r="A17" s="29" t="n">
         <x:v>46292</x:v>
       </x:c>
-      <x:c r="B17" s="13" t="str">
+      <x:c r="B17" s="18" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C17" s="18"/>
-      <x:c r="D17" s="18"/>
-      <x:c r="E17" s="24" t="str">
+      <x:c r="C17" s="24"/>
+      <x:c r="D17" s="24"/>
+      <x:c r="E17" s="24"/>
+      <x:c r="F17" s="24"/>
+      <x:c r="G17" s="24"/>
+      <x:c r="H17" s="24"/>
+      <x:c r="I17" s="30" t="str">
         <x:v>주은성</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="22" customHeight="1">
-      <x:c r="A18" s="23" t="n">
+    <x:row r="18" ht="25" customHeight="1">
+      <x:c r="A18" s="29" t="n">
         <x:v>46298</x:v>
       </x:c>
-      <x:c r="B18" s="13" t="str">
+      <x:c r="B18" s="18" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C18" s="18"/>
-      <x:c r="D18" s="18"/>
-      <x:c r="E18" s="24" t="str">
+      <x:c r="C18" s="24"/>
+      <x:c r="D18" s="24"/>
+      <x:c r="E18" s="24"/>
+      <x:c r="F18" s="24"/>
+      <x:c r="G18" s="24"/>
+      <x:c r="H18" s="24"/>
+      <x:c r="I18" s="30" t="str">
         <x:v>주은성</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="22" customHeight="1">
-      <x:c r="A19" s="23" t="n">
+    <x:row r="19" ht="25" customHeight="1">
+      <x:c r="A19" s="29" t="n">
         <x:v>46298</x:v>
       </x:c>
-      <x:c r="B19" s="13" t="str">
+      <x:c r="B19" s="18" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C19" s="18"/>
-      <x:c r="D19" s="18"/>
-      <x:c r="E19" s="24" t="str">
+      <x:c r="C19" s="24"/>
+      <x:c r="D19" s="24"/>
+      <x:c r="E19" s="24"/>
+      <x:c r="F19" s="24"/>
+      <x:c r="G19" s="24"/>
+      <x:c r="H19" s="24"/>
+      <x:c r="I19" s="30" t="str">
         <x:v>이상</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="22" customHeight="1">
-      <x:c r="A20" s="23" t="n">
+    <x:row r="20" ht="25" customHeight="1">
+      <x:c r="A20" s="29" t="n">
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="B20" s="13" t="str">
+      <x:c r="B20" s="18" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C20" s="18"/>
-      <x:c r="D20" s="18"/>
-      <x:c r="E20" s="24" t="str">
+      <x:c r="C20" s="24"/>
+      <x:c r="D20" s="24"/>
+      <x:c r="E20" s="24"/>
+      <x:c r="F20" s="24"/>
+      <x:c r="G20" s="24"/>
+      <x:c r="H20" s="24"/>
+      <x:c r="I20" s="30" t="str">
         <x:v>문권기</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="22" customHeight="1">
-      <x:c r="A21" s="25" t="n">
+    <x:row r="21" ht="25" customHeight="1">
+      <x:c r="A21" s="31" t="n">
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="B21" s="26" t="str">
+      <x:c r="B21" s="32" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C21" s="27"/>
-      <x:c r="D21" s="27"/>
-      <x:c r="E21" s="28" t="str">
+      <x:c r="C21" s="33"/>
+      <x:c r="D21" s="33"/>
+      <x:c r="E21" s="33"/>
+      <x:c r="F21" s="33"/>
+      <x:c r="G21" s="33"/>
+      <x:c r="H21" s="33"/>
+      <x:c r="I21" s="34" t="str">
         <x:v>이상</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="K1:M1"/>
+    <x:mergeCell ref="K2:M6"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26881e6e0c8b46fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72081ec6a6a1488d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>